<commit_message>
ultradata: append 5 rows [2026-03-26]
</commit_message>
<xml_diff>
--- a/ultradata.xlsx
+++ b/ultradata.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -698,6 +698,241 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Whole Fish</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>fish_seafood</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>whole_fish</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>img_000170.png</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1HYsd8o24FoQ6-pxI_w3iLo8U0z0uvDZT</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>10FuamWRoIrDjYVzzyLJV9-UZZ8rAxffn</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1HYsd8o24FoQ6-pxI_w3iLo8U0z0uvDZT&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/10FuamWRoIrDjYVzzyLJV9-UZZ8rAxffn=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Crab</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>fish_seafood</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>crab</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>img_000176.png</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1FO-EsfgudO67EdeYe5WpF7gV0E5GGy1Q</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>1SJGL1oz5nA4miHHiLB3l85Ya2ueo8j3K</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1FO-EsfgudO67EdeYe5WpF7gV0E5GGy1Q&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1SJGL1oz5nA4miHHiLB3l85Ya2ueo8j3K=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Crab</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>fish_seafood</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>crab</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>img_000180.png</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1EFf0kILXifNQtwTA7Dxde48G9LUPipZR</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>1wIRj9irDqLJAoz1CbP4o5j_o8PIyPAGX</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1EFf0kILXifNQtwTA7Dxde48G9LUPipZR&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1wIRj9irDqLJAoz1CbP4o5j_o8PIyPAGX=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Whole Fish</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>fish_seafood</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>whole_fish</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>img_000195.png</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>1s5Irm3xQagAjZrng7L_FaNfP_kcnwZII</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>1w7JeNCZInfEKWNu7uVzC7olfHUvek7gJ</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1s5Irm3xQagAjZrng7L_FaNfP_kcnwZII&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1w7JeNCZInfEKWNu7uVzC7olfHUvek7gJ=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Whole Fish</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>fish_seafood</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>whole_fish</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>img_000216.png</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>1GS4C-uQhFKHbhewPow15AHMiEExKnBIv</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>1G1BEcQ91q1LPdrHPC4cgBjHAGTbFvDKJ</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1GS4C-uQhFKHbhewPow15AHMiEExKnBIv&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1G1BEcQ91q1LPdrHPC4cgBjHAGTbFvDKJ=s800</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
ultradata: append 5 rows [2026-03-29]
</commit_message>
<xml_diff>
--- a/ultradata.xlsx
+++ b/ultradata.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I811"/>
+  <dimension ref="A1:I816"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38533,6 +38533,241 @@
         </is>
       </c>
     </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>Cow</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>animals</t>
+        </is>
+      </c>
+      <c r="D812" t="inlineStr">
+        <is>
+          <t>cow</t>
+        </is>
+      </c>
+      <c r="E812" t="inlineStr">
+        <is>
+          <t>img_004767.png</t>
+        </is>
+      </c>
+      <c r="F812" t="inlineStr">
+        <is>
+          <t>1tI-RaaoZTlMckm-veig0-ZL1iWeqtdJi</t>
+        </is>
+      </c>
+      <c r="G812" t="inlineStr">
+        <is>
+          <t>1ebdvs99I4yuOI6rf0gw23j6e_y_47t-k</t>
+        </is>
+      </c>
+      <c r="H812" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1tI-RaaoZTlMckm-veig0-ZL1iWeqtdJi&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I812" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1ebdvs99I4yuOI6rf0gw23j6e_y_47t-k=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>Cow</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>animals</t>
+        </is>
+      </c>
+      <c r="D813" t="inlineStr">
+        <is>
+          <t>cow</t>
+        </is>
+      </c>
+      <c r="E813" t="inlineStr">
+        <is>
+          <t>img_002865.png</t>
+        </is>
+      </c>
+      <c r="F813" t="inlineStr">
+        <is>
+          <t>1Ulq4MXUhnPwv0KVT74YaqYDQ5757_VJu</t>
+        </is>
+      </c>
+      <c r="G813" t="inlineStr">
+        <is>
+          <t>1L_AdNaVWOCjwY7bJd5I_BsODl_dkelf8</t>
+        </is>
+      </c>
+      <c r="H813" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1Ulq4MXUhnPwv0KVT74YaqYDQ5757_VJu&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I813" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1L_AdNaVWOCjwY7bJd5I_BsODl_dkelf8=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>Cow</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>animals</t>
+        </is>
+      </c>
+      <c r="D814" t="inlineStr">
+        <is>
+          <t>cow</t>
+        </is>
+      </c>
+      <c r="E814" t="inlineStr">
+        <is>
+          <t>img_005019.png</t>
+        </is>
+      </c>
+      <c r="F814" t="inlineStr">
+        <is>
+          <t>1fhNYtz8c-ALWm4NLhz5UwwGUfnUWWeq-</t>
+        </is>
+      </c>
+      <c r="G814" t="inlineStr">
+        <is>
+          <t>1DVv8hmHNIiJbjp35uh0fHFJx9ZUWpcJc</t>
+        </is>
+      </c>
+      <c r="H814" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1fhNYtz8c-ALWm4NLhz5UwwGUfnUWWeq-&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I814" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1DVv8hmHNIiJbjp35uh0fHFJx9ZUWpcJc=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>Cow</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>animals</t>
+        </is>
+      </c>
+      <c r="D815" t="inlineStr">
+        <is>
+          <t>cow</t>
+        </is>
+      </c>
+      <c r="E815" t="inlineStr">
+        <is>
+          <t>img_002235.png</t>
+        </is>
+      </c>
+      <c r="F815" t="inlineStr">
+        <is>
+          <t>1oaMq7N2LrYKDSQAwmKEzW2qFvJJAAVTm</t>
+        </is>
+      </c>
+      <c r="G815" t="inlineStr">
+        <is>
+          <t>114AXsx2c3KmcBiuREz7Sf4xSFAKNCTcw</t>
+        </is>
+      </c>
+      <c r="H815" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1oaMq7N2LrYKDSQAwmKEzW2qFvJJAAVTm&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I815" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/114AXsx2c3KmcBiuREz7Sf4xSFAKNCTcw=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>Cow</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>animals</t>
+        </is>
+      </c>
+      <c r="D816" t="inlineStr">
+        <is>
+          <t>cow</t>
+        </is>
+      </c>
+      <c r="E816" t="inlineStr">
+        <is>
+          <t>img_001834.png</t>
+        </is>
+      </c>
+      <c r="F816" t="inlineStr">
+        <is>
+          <t>1kkBw9rkcSe4AQ1fHSpo1iBQlU3Bdbrsd</t>
+        </is>
+      </c>
+      <c r="G816" t="inlineStr">
+        <is>
+          <t>18cRE47PLrAx-K_B1LoM9SXpQjg2OEL-P</t>
+        </is>
+      </c>
+      <c r="H816" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1kkBw9rkcSe4AQ1fHSpo1iBQlU3Bdbrsd&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I816" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/18cRE47PLrAx-K_B1LoM9SXpQjg2OEL-P=s800</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
ultradata: append 10 rows [2026-03-29]
</commit_message>
<xml_diff>
--- a/ultradata.xlsx
+++ b/ultradata.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I816"/>
+  <dimension ref="A1:I826"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38768,6 +38768,476 @@
         </is>
       </c>
     </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>Admissions Open</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>ADMISSIONS &amp; ENROLLMENT</t>
+        </is>
+      </c>
+      <c r="D817" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E817" t="inlineStr">
+        <is>
+          <t>admissions_open_01.png</t>
+        </is>
+      </c>
+      <c r="F817" t="inlineStr">
+        <is>
+          <t>1mnuZXZ10jVrRdqJMGGCfxMdq5LKztUG9</t>
+        </is>
+      </c>
+      <c r="G817" t="inlineStr">
+        <is>
+          <t>1rk3g-cQinPlvWe2yiz1jpdHUFSPrcSUI</t>
+        </is>
+      </c>
+      <c r="H817" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1mnuZXZ10jVrRdqJMGGCfxMdq5LKztUG9&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I817" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1rk3g-cQinPlvWe2yiz1jpdHUFSPrcSUI=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>Admissions Open</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>ADMISSIONS &amp; ENROLLMENT</t>
+        </is>
+      </c>
+      <c r="D818" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E818" t="inlineStr">
+        <is>
+          <t>admissions_open_02.png</t>
+        </is>
+      </c>
+      <c r="F818" t="inlineStr">
+        <is>
+          <t>1F_1GoqLxrLrqFaBNrSbg9jkEnWJYiYn7</t>
+        </is>
+      </c>
+      <c r="G818" t="inlineStr">
+        <is>
+          <t>19hZZK_PockuRQJ2j57M94p8mjsWf9dt4</t>
+        </is>
+      </c>
+      <c r="H818" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1F_1GoqLxrLrqFaBNrSbg9jkEnWJYiYn7&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I818" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/19hZZK_PockuRQJ2j57M94p8mjsWf9dt4=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>Admissions Open</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>ADMISSIONS &amp; ENROLLMENT</t>
+        </is>
+      </c>
+      <c r="D819" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E819" t="inlineStr">
+        <is>
+          <t>admissions_open_03.png</t>
+        </is>
+      </c>
+      <c r="F819" t="inlineStr">
+        <is>
+          <t>17GFl6311_qHtNndqr1rQEdZ2VkviiYqj</t>
+        </is>
+      </c>
+      <c r="G819" t="inlineStr">
+        <is>
+          <t>1QLp3vlboHmQlgxyln3q3nmZc6AEbXrJE</t>
+        </is>
+      </c>
+      <c r="H819" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=17GFl6311_qHtNndqr1rQEdZ2VkviiYqj&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I819" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1QLp3vlboHmQlgxyln3q3nmZc6AEbXrJE=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>Admissions Open</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>ADMISSIONS &amp; ENROLLMENT</t>
+        </is>
+      </c>
+      <c r="D820" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E820" t="inlineStr">
+        <is>
+          <t>admissions_open_04.png</t>
+        </is>
+      </c>
+      <c r="F820" t="inlineStr">
+        <is>
+          <t>1G_IImrTZ2WnMhLqM9XAKgUjbpp6ZPUhm</t>
+        </is>
+      </c>
+      <c r="G820" t="inlineStr">
+        <is>
+          <t>1xOVAakFq4GhjONyk7twwDD6arkx5qukD</t>
+        </is>
+      </c>
+      <c r="H820" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1G_IImrTZ2WnMhLqM9XAKgUjbpp6ZPUhm&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I820" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1xOVAakFq4GhjONyk7twwDD6arkx5qukD=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>Admissions Open</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>ADMISSIONS &amp; ENROLLMENT</t>
+        </is>
+      </c>
+      <c r="D821" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E821" t="inlineStr">
+        <is>
+          <t>admissions_open_05.png</t>
+        </is>
+      </c>
+      <c r="F821" t="inlineStr">
+        <is>
+          <t>11QvgPCcQ6-sbAM_1xYjujIIqh_k8Do7y</t>
+        </is>
+      </c>
+      <c r="G821" t="inlineStr">
+        <is>
+          <t>1ucdamz3IHFAIUr_6qCxpfnN7qCxoyUn-</t>
+        </is>
+      </c>
+      <c r="H821" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=11QvgPCcQ6-sbAM_1xYjujIIqh_k8Do7y&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I821" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1ucdamz3IHFAIUr_6qCxpfnN7qCxoyUn-=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>Admissions Open</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>ADMISSIONS &amp; ENROLLMENT</t>
+        </is>
+      </c>
+      <c r="D822" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E822" t="inlineStr">
+        <is>
+          <t>admissions_open_06.png</t>
+        </is>
+      </c>
+      <c r="F822" t="inlineStr">
+        <is>
+          <t>1GmgoMUYvYB9FT-XM590wBo5doSfF9qJ5</t>
+        </is>
+      </c>
+      <c r="G822" t="inlineStr">
+        <is>
+          <t>1XcFO8EpIXSiMP2qrYRalh0JLz4TDVg9n</t>
+        </is>
+      </c>
+      <c r="H822" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1GmgoMUYvYB9FT-XM590wBo5doSfF9qJ5&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I822" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1XcFO8EpIXSiMP2qrYRalh0JLz4TDVg9n=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>Admissions Open</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>ADMISSIONS &amp; ENROLLMENT</t>
+        </is>
+      </c>
+      <c r="D823" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E823" t="inlineStr">
+        <is>
+          <t>admissions_open_07.png</t>
+        </is>
+      </c>
+      <c r="F823" t="inlineStr">
+        <is>
+          <t>1sHUwqgsx2xMb316BmRUd_45kNX3Q1c_q</t>
+        </is>
+      </c>
+      <c r="G823" t="inlineStr">
+        <is>
+          <t>1AAb7jHeOE_7y_Phs310wTxKMlp4hyAzD</t>
+        </is>
+      </c>
+      <c r="H823" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1sHUwqgsx2xMb316BmRUd_45kNX3Q1c_q&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I823" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1AAb7jHeOE_7y_Phs310wTxKMlp4hyAzD=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>Admissions Open</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>ADMISSIONS &amp; ENROLLMENT</t>
+        </is>
+      </c>
+      <c r="D824" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E824" t="inlineStr">
+        <is>
+          <t>admissions_open_08.png</t>
+        </is>
+      </c>
+      <c r="F824" t="inlineStr">
+        <is>
+          <t>1YTiCi7bbEUQDh65Bjv5HxYtTY7hGdwwC</t>
+        </is>
+      </c>
+      <c r="G824" t="inlineStr">
+        <is>
+          <t>1rR2apc_EF37QmAPLTupydohX-KW2_e-2</t>
+        </is>
+      </c>
+      <c r="H824" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1YTiCi7bbEUQDh65Bjv5HxYtTY7hGdwwC&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I824" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1rR2apc_EF37QmAPLTupydohX-KW2_e-2=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>Admissions Open</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>ADMISSIONS &amp; ENROLLMENT</t>
+        </is>
+      </c>
+      <c r="D825" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E825" t="inlineStr">
+        <is>
+          <t>admissions_open_09.png</t>
+        </is>
+      </c>
+      <c r="F825" t="inlineStr">
+        <is>
+          <t>1HOhZYu_ry3st4VE9GSm8ZrGuGdLhLfvw</t>
+        </is>
+      </c>
+      <c r="G825" t="inlineStr">
+        <is>
+          <t>1jk89wiYWgTL77au5kyRNoZBKfXYKGtCW</t>
+        </is>
+      </c>
+      <c r="H825" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1HOhZYu_ry3st4VE9GSm8ZrGuGdLhLfvw&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I825" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1jk89wiYWgTL77au5kyRNoZBKfXYKGtCW=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>Admissions Open</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>ADMISSIONS &amp; ENROLLMENT</t>
+        </is>
+      </c>
+      <c r="D826" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E826" t="inlineStr">
+        <is>
+          <t>admissions_open_10.png</t>
+        </is>
+      </c>
+      <c r="F826" t="inlineStr">
+        <is>
+          <t>1_8jJiTLWdmqxd-zm-2_E0ckK-6faLEsg</t>
+        </is>
+      </c>
+      <c r="G826" t="inlineStr">
+        <is>
+          <t>1-RLoyBJnpI3zsGDarCC9fagPgRVLL7lm</t>
+        </is>
+      </c>
+      <c r="H826" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1_8jJiTLWdmqxd-zm-2_E0ckK-6faLEsg&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I826" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1-RLoyBJnpI3zsGDarCC9fagPgRVLL7lm=s800</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
ultradata: zimage-logo append 5 rows [2026-03-31]
</commit_message>
<xml_diff>
--- a/ultradata.xlsx
+++ b/ultradata.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1126"/>
+  <dimension ref="A1:I1131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53338,6 +53338,241 @@
         </is>
       </c>
     </row>
+    <row r="1127">
+      <c r="A1127" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B1127" t="inlineStr">
+        <is>
+          <t>Important Notice</t>
+        </is>
+      </c>
+      <c r="C1127" t="inlineStr">
+        <is>
+          <t>ANNOUNCEMENTS</t>
+        </is>
+      </c>
+      <c r="D1127" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E1127" t="inlineStr">
+        <is>
+          <t>important_notice_11.png</t>
+        </is>
+      </c>
+      <c r="F1127" t="inlineStr">
+        <is>
+          <t>1VW6D5vht2gCdUnC89IDC50xUYrzCAmdW</t>
+        </is>
+      </c>
+      <c r="G1127" t="inlineStr">
+        <is>
+          <t>1_yPVDqhuqsBYHky8S4BF_G6dx9LrQo48</t>
+        </is>
+      </c>
+      <c r="H1127" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1VW6D5vht2gCdUnC89IDC50xUYrzCAmdW&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I1127" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1_yPVDqhuqsBYHky8S4BF_G6dx9LrQo48=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B1128" t="inlineStr">
+        <is>
+          <t>Important Notice</t>
+        </is>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>ANNOUNCEMENTS</t>
+        </is>
+      </c>
+      <c r="D1128" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E1128" t="inlineStr">
+        <is>
+          <t>important_notice_12.png</t>
+        </is>
+      </c>
+      <c r="F1128" t="inlineStr">
+        <is>
+          <t>1MybH1NxJ9zB4JNcIZ03UlYchIhE7z5PK</t>
+        </is>
+      </c>
+      <c r="G1128" t="inlineStr">
+        <is>
+          <t>1kNGi66R0hrLQu4cssyR9QSPoU-Up3G1z</t>
+        </is>
+      </c>
+      <c r="H1128" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1MybH1NxJ9zB4JNcIZ03UlYchIhE7z5PK&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I1128" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1kNGi66R0hrLQu4cssyR9QSPoU-Up3G1z=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B1129" t="inlineStr">
+        <is>
+          <t>Important Notice</t>
+        </is>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>ANNOUNCEMENTS</t>
+        </is>
+      </c>
+      <c r="D1129" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E1129" t="inlineStr">
+        <is>
+          <t>important_notice_13.png</t>
+        </is>
+      </c>
+      <c r="F1129" t="inlineStr">
+        <is>
+          <t>17qYPalQFyMWas4PPGUZPN0nLbLxjSPax</t>
+        </is>
+      </c>
+      <c r="G1129" t="inlineStr">
+        <is>
+          <t>1kLn0LOk9iykbYjpz4MwFo6tE_n6BOdPe</t>
+        </is>
+      </c>
+      <c r="H1129" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=17qYPalQFyMWas4PPGUZPN0nLbLxjSPax&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I1129" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1kLn0LOk9iykbYjpz4MwFo6tE_n6BOdPe=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B1130" t="inlineStr">
+        <is>
+          <t>Important Notice</t>
+        </is>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>ANNOUNCEMENTS</t>
+        </is>
+      </c>
+      <c r="D1130" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E1130" t="inlineStr">
+        <is>
+          <t>important_notice_14.png</t>
+        </is>
+      </c>
+      <c r="F1130" t="inlineStr">
+        <is>
+          <t>17kicJoUHgD-FDWzD8tYX6O_gpJqu9cbx</t>
+        </is>
+      </c>
+      <c r="G1130" t="inlineStr">
+        <is>
+          <t>1lXIe3sPUn8-rPXxr96lEjXF-zf5rUa8F</t>
+        </is>
+      </c>
+      <c r="H1130" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=17kicJoUHgD-FDWzD8tYX6O_gpJqu9cbx&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I1130" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1lXIe3sPUn8-rPXxr96lEjXF-zf5rUa8F=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B1131" t="inlineStr">
+        <is>
+          <t>Important Notice</t>
+        </is>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>ANNOUNCEMENTS</t>
+        </is>
+      </c>
+      <c r="D1131" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E1131" t="inlineStr">
+        <is>
+          <t>important_notice_15.png</t>
+        </is>
+      </c>
+      <c r="F1131" t="inlineStr">
+        <is>
+          <t>1TlmtCfT26s4oQVDmXEikY8zTMu9aG3Lc</t>
+        </is>
+      </c>
+      <c r="G1131" t="inlineStr">
+        <is>
+          <t>1rq0NYeSYXJRlpTmkxNGUKnW6r8Dl1zeu</t>
+        </is>
+      </c>
+      <c r="H1131" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1TlmtCfT26s4oQVDmXEikY8zTMu9aG3Lc&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I1131" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1rq0NYeSYXJRlpTmkxNGUKnW6r8Dl1zeu=s800</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
ultradata: append 10 rows [2026-04-05]
</commit_message>
<xml_diff>
--- a/ultradata.xlsx
+++ b/ultradata.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1146"/>
+  <dimension ref="A1:I1156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54278,6 +54278,476 @@
         </is>
       </c>
     </row>
+    <row r="1147">
+      <c r="A1147" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>FRUITS</t>
+        </is>
+      </c>
+      <c r="D1147" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E1147" t="inlineStr">
+        <is>
+          <t>banana_01.png</t>
+        </is>
+      </c>
+      <c r="F1147" t="inlineStr">
+        <is>
+          <t>1Qfn6UK37EV28qEyu6_sO7M8V8MP_PxKi</t>
+        </is>
+      </c>
+      <c r="G1147" t="inlineStr">
+        <is>
+          <t>1cgFNEmV9UDRjCj4jW3TgRuYsyRN0c-6G</t>
+        </is>
+      </c>
+      <c r="H1147" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1Qfn6UK37EV28qEyu6_sO7M8V8MP_PxKi&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I1147" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1cgFNEmV9UDRjCj4jW3TgRuYsyRN0c-6G=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>FRUITS</t>
+        </is>
+      </c>
+      <c r="D1148" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E1148" t="inlineStr">
+        <is>
+          <t>banana_02.png</t>
+        </is>
+      </c>
+      <c r="F1148" t="inlineStr">
+        <is>
+          <t>1FR6pPMfLhO3KOSVz7gJ3ylcyNKTDMp1o</t>
+        </is>
+      </c>
+      <c r="G1148" t="inlineStr">
+        <is>
+          <t>1hEUBC4T5Uuu0TqdAQdZb6GD5ithUIrep</t>
+        </is>
+      </c>
+      <c r="H1148" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1FR6pPMfLhO3KOSVz7gJ3ylcyNKTDMp1o&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I1148" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1hEUBC4T5Uuu0TqdAQdZb6GD5ithUIrep=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>FRUITS</t>
+        </is>
+      </c>
+      <c r="D1149" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E1149" t="inlineStr">
+        <is>
+          <t>banana_03.png</t>
+        </is>
+      </c>
+      <c r="F1149" t="inlineStr">
+        <is>
+          <t>1HlfG5IEy06wYiO0-OcImzC0ZbQgPmfS5</t>
+        </is>
+      </c>
+      <c r="G1149" t="inlineStr">
+        <is>
+          <t>1MJcLDPW9QCYpyIiZdFLio12euuXkZ9Qo</t>
+        </is>
+      </c>
+      <c r="H1149" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1HlfG5IEy06wYiO0-OcImzC0ZbQgPmfS5&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I1149" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1MJcLDPW9QCYpyIiZdFLio12euuXkZ9Qo=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B1150" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>FRUITS</t>
+        </is>
+      </c>
+      <c r="D1150" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E1150" t="inlineStr">
+        <is>
+          <t>banana_04.png</t>
+        </is>
+      </c>
+      <c r="F1150" t="inlineStr">
+        <is>
+          <t>12-7q9OP5U_iKJKWlEbusC6OMv0gsAkUO</t>
+        </is>
+      </c>
+      <c r="G1150" t="inlineStr">
+        <is>
+          <t>1yYIvik9y83r5X14dqaefQ4kY1-Bmx6s3</t>
+        </is>
+      </c>
+      <c r="H1150" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=12-7q9OP5U_iKJKWlEbusC6OMv0gsAkUO&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I1150" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1yYIvik9y83r5X14dqaefQ4kY1-Bmx6s3=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B1151" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>FRUITS</t>
+        </is>
+      </c>
+      <c r="D1151" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E1151" t="inlineStr">
+        <is>
+          <t>banana_05.png</t>
+        </is>
+      </c>
+      <c r="F1151" t="inlineStr">
+        <is>
+          <t>1E8NkOodpXszbA-5emJ3J0k3Ku1YolSq0</t>
+        </is>
+      </c>
+      <c r="G1151" t="inlineStr">
+        <is>
+          <t>1jjeXKt6a3YABNSZukw8e_C1JzO5X68aM</t>
+        </is>
+      </c>
+      <c r="H1151" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1E8NkOodpXszbA-5emJ3J0k3Ku1YolSq0&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I1151" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1jjeXKt6a3YABNSZukw8e_C1JzO5X68aM=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B1152" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>FRUITS</t>
+        </is>
+      </c>
+      <c r="D1152" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E1152" t="inlineStr">
+        <is>
+          <t>banana_06.png</t>
+        </is>
+      </c>
+      <c r="F1152" t="inlineStr">
+        <is>
+          <t>1OjyYyVJwhz0TSaPsuOEZz-XFJcUH-bKk</t>
+        </is>
+      </c>
+      <c r="G1152" t="inlineStr">
+        <is>
+          <t>1Sb4Aq5gwIpwIKYBjfpP1leki0Rrpvkp8</t>
+        </is>
+      </c>
+      <c r="H1152" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1OjyYyVJwhz0TSaPsuOEZz-XFJcUH-bKk&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I1152" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1Sb4Aq5gwIpwIKYBjfpP1leki0Rrpvkp8=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>FRUITS</t>
+        </is>
+      </c>
+      <c r="D1153" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E1153" t="inlineStr">
+        <is>
+          <t>banana_07.png</t>
+        </is>
+      </c>
+      <c r="F1153" t="inlineStr">
+        <is>
+          <t>1NAQu_BiojZMRfUm3sCtLuR6x5_2Kbnbu</t>
+        </is>
+      </c>
+      <c r="G1153" t="inlineStr">
+        <is>
+          <t>1HJV-5tdeU0GW_z-cJYiKlsFSDXgLEpYH</t>
+        </is>
+      </c>
+      <c r="H1153" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1NAQu_BiojZMRfUm3sCtLuR6x5_2Kbnbu&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I1153" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1HJV-5tdeU0GW_z-cJYiKlsFSDXgLEpYH=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>FRUITS</t>
+        </is>
+      </c>
+      <c r="D1154" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E1154" t="inlineStr">
+        <is>
+          <t>banana_08.png</t>
+        </is>
+      </c>
+      <c r="F1154" t="inlineStr">
+        <is>
+          <t>1vMwNnxLURjRMqne6WkvxsmiE8gAVRjee</t>
+        </is>
+      </c>
+      <c r="G1154" t="inlineStr">
+        <is>
+          <t>1L7A7XrMVADSYRqN-QSd9KpDxdGHVnkTI</t>
+        </is>
+      </c>
+      <c r="H1154" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1vMwNnxLURjRMqne6WkvxsmiE8gAVRjee&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I1154" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1L7A7XrMVADSYRqN-QSd9KpDxdGHVnkTI=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>FRUITS</t>
+        </is>
+      </c>
+      <c r="D1155" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E1155" t="inlineStr">
+        <is>
+          <t>banana_09.png</t>
+        </is>
+      </c>
+      <c r="F1155" t="inlineStr">
+        <is>
+          <t>1DxGf4SosZ8wjXt_7fjC9J5JrciTnRmZC</t>
+        </is>
+      </c>
+      <c r="G1155" t="inlineStr">
+        <is>
+          <t>19WIMVFE7RbvpZJZudEj_nM4gOtsq0cGg</t>
+        </is>
+      </c>
+      <c r="H1155" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1DxGf4SosZ8wjXt_7fjC9J5JrciTnRmZC&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I1155" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/19WIMVFE7RbvpZJZudEj_nM4gOtsq0cGg=s800</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>FRUITS</t>
+        </is>
+      </c>
+      <c r="D1156" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E1156" t="inlineStr">
+        <is>
+          <t>banana_10.png</t>
+        </is>
+      </c>
+      <c r="F1156" t="inlineStr">
+        <is>
+          <t>1Nb5tfkVJhfr3tZPtx6LfIlKoO4Bn-AHg</t>
+        </is>
+      </c>
+      <c r="G1156" t="inlineStr">
+        <is>
+          <t>1iLVFGiGuSrErxMTDl-TC5CFfcMemzxYV</t>
+        </is>
+      </c>
+      <c r="H1156" t="inlineStr">
+        <is>
+          <t>https://drive.usercontent.google.com/download?id=1Nb5tfkVJhfr3tZPtx6LfIlKoO4Bn-AHg&amp;export=download&amp;authuser=0</t>
+        </is>
+      </c>
+      <c r="I1156" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/d/1iLVFGiGuSrErxMTDl-TC5CFfcMemzxYV=s800</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>